<commit_message>
Data: 20/02/2026 - Hora: 00:00:00,00
</commit_message>
<xml_diff>
--- a/ksoft/_bakas/Papeis DP E FF.xlsx
+++ b/ksoft/_bakas/Papeis DP E FF.xlsx
@@ -5949,8 +5949,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F97EE73F6824CB4CBC81148F022C7122" ma:contentTypeVersion="19" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="c135dfd5689eb1f41c942b6de29d974a">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d196706a-de7c-4813-9c30-935ec1d4cc5d" xmlns:ns3="dd292427-de11-427f-a4cf-93902db2c621" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f598600a6f7a583361fdb2bebd14dd7" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F97EE73F6824CB4CBC81148F022C7122" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="3acbdff660be4f41504a7377bd00bfbe">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d196706a-de7c-4813-9c30-935ec1d4cc5d" xmlns:ns3="dd292427-de11-427f-a4cf-93902db2c621" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3d165de6d9d878c1143ab435ba51092c" ns2:_="" ns3:_="">
     <xsd:import namespace="d196706a-de7c-4813-9c30-935ec1d4cc5d"/>
     <xsd:import namespace="dd292427-de11-427f-a4cf-93902db2c621"/>
     <xsd:element name="properties">
@@ -6040,7 +6040,7 @@
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de Imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8e0251ee-03ea-4cdd-a84b-a8795fd5a69c" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8e0251ee-03ea-4cdd-a84b-a8795fd5a69c" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -6066,7 +6066,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="dd292427-de11-427f-a4cf-93902db2c621" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Partilhado Com" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Compartilhado com" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -6085,7 +6085,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Detalhes de Partilhado Com" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Detalhes de Compartilhado Com" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -6224,13 +6224,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08F7D190-6674-4586-AE0F-886E37E6F661}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6981508A-992C-49E2-9C1A-FBB12E3B6EAB}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28B8F830-4310-4B6C-B334-3514634DA37C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4B18E3A-A801-45CD-8B32-74E329DEE507}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{274DFCD1-B629-40D4-88D0-54B245E78E5D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A85C37E0-2B6A-4F3F-AA5C-C4D94BC2EF8E}"/>
 </file>
</xml_diff>

<commit_message>
Data: 06/03/2026 - Hora: 00:00:00,00
</commit_message>
<xml_diff>
--- a/ksoft/_bakas/Papeis DP E FF.xlsx
+++ b/ksoft/_bakas/Papeis DP E FF.xlsx
@@ -5949,8 +5949,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F97EE73F6824CB4CBC81148F022C7122" ma:contentTypeVersion="19" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="3acbdff660be4f41504a7377bd00bfbe">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d196706a-de7c-4813-9c30-935ec1d4cc5d" xmlns:ns3="dd292427-de11-427f-a4cf-93902db2c621" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3d165de6d9d878c1143ab435ba51092c" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100F97EE73F6824CB4CBC81148F022C7122" ma:contentTypeVersion="19" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="c135dfd5689eb1f41c942b6de29d974a">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="d196706a-de7c-4813-9c30-935ec1d4cc5d" xmlns:ns3="dd292427-de11-427f-a4cf-93902db2c621" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f598600a6f7a583361fdb2bebd14dd7" ns2:_="" ns3:_="">
     <xsd:import namespace="d196706a-de7c-4813-9c30-935ec1d4cc5d"/>
     <xsd:import namespace="dd292427-de11-427f-a4cf-93902db2c621"/>
     <xsd:element name="properties">
@@ -6040,7 +6040,7 @@
         <xsd:restriction base="dms:Unknown"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8e0251ee-03ea-4cdd-a84b-a8795fd5a69c" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="21" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de Imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="8e0251ee-03ea-4cdd-a84b-a8795fd5a69c" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -6066,7 +6066,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="dd292427-de11-427f-a4cf-93902db2c621" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Compartilhado com" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Partilhado Com" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -6085,7 +6085,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Detalhes de Compartilhado Com" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Detalhes de Partilhado Com" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -6224,13 +6224,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6981508A-992C-49E2-9C1A-FBB12E3B6EAB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD4DBBC2-5F5C-4F50-99A5-AB87CD0D3E92}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E4B18E3A-A801-45CD-8B32-74E329DEE507}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DF1558FD-D019-4944-8CBD-D6C99752AFD6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A85C37E0-2B6A-4F3F-AA5C-C4D94BC2EF8E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ECF1B028-EE73-49CA-B13E-3FE4EE728FCB}"/>
 </file>
</xml_diff>